<commit_message>
Add 2016-2018 tax-credit reports (scanned, transcribed)
The 2016, 2017, and 2018 CDC Tax Credit reports from Ben's email are
image-only scans with no text layer. Rendered the participation tables
and transcribed them into data/taxcredit_scanned.csv, which the parser
now merges. Participation timelines are contiguous 2015-2020, confirming
continuous enrollment and catching gaps (e.g. Allegheny West absent 2018).
All six source report PDFs are hosted locally and linked from each org's
tax-credit card. 251 participation rows across 6 report years.
</commit_message>
<xml_diff>
--- a/output/corridor_dataset.xlsx
+++ b/output/corridor_dataset.xlsx
@@ -683,11 +683,7 @@
       <c r="K4" t="n">
         <v>100000</v>
       </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="L4" t="inlineStr"/>
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="inlineStr">
         <is>
@@ -26146,7 +26142,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D127"/>
+  <dimension ref="A1:D252"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -26856,7 +26852,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C44" t="n">
         <v>2012</v>
@@ -26868,11 +26864,11 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Asociaciόn Puertorriqueños En Marcha, Inc</t>
+          <t>Asociación Puertorriqueños En Marcha Inc</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C45" t="n">
         <v>2015</v>
@@ -26884,11 +26880,11 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Beech Interplex, Inc.</t>
+          <t>Beech Interplex Inc.</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C46" t="n">
         <v>2013</v>
@@ -26904,7 +26900,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C47" t="n">
         <v>2012</v>
@@ -26920,7 +26916,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C48" t="n">
         <v>2013</v>
@@ -26932,11 +26928,11 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Common Market Philadelphia, Inc., HFI</t>
+          <t>Common Market Philadelphia Inc.</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C49" t="n">
         <v>2013</v>
@@ -26948,11 +26944,11 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Community Design Collaborative, NPI</t>
+          <t>Community Design Collaborative</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C50" t="n">
         <v>2012</v>
@@ -26964,14 +26960,14 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Delaware River City Corporation (DRCC)</t>
+          <t>Delaware River City Corporation (Frmly Delaware Riverfront Renaissance Corp.)</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C51" t="n">
-        <v>2017</v>
+        <v>2010</v>
       </c>
       <c r="D51" t="n">
         <v>100000</v>
@@ -26984,7 +26980,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C52" t="n">
         <v>2013</v>
@@ -27000,7 +26996,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C53" t="n">
         <v>2012</v>
@@ -27016,7 +27012,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C54" t="n">
         <v>2013</v>
@@ -27032,7 +27028,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C55" t="n">
         <v>2014</v>
@@ -27048,7 +27044,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C56" t="n">
         <v>2015</v>
@@ -27064,7 +27060,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C57" t="n">
         <v>2012</v>
@@ -27076,30 +27072,30 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Germantown United Community Development Corporation</t>
+          <t>HACE aka Hispanic Assoc. of Contractors &amp; Enterprises</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C58" t="n">
-        <v>2019</v>
+        <v>2013</v>
       </c>
       <c r="D58" t="n">
-        <v>100000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>HACE aka Hispanic Assoc. of Contractors &amp; Enterprises</t>
+          <t>Impact Services Corporation</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C59" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="D59" t="n">
         <v>85000</v>
@@ -27108,43 +27104,43 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Impact Services Corporation</t>
+          <t>Manayunk Development Corporation</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C60" t="n">
-        <v>2012</v>
+        <v>2010</v>
       </c>
       <c r="D60" t="n">
-        <v>85000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Manayunk Development Corporation</t>
+          <t>Mayfair Community Development Corporation</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C61" t="n">
-        <v>2010</v>
+        <v>2013</v>
       </c>
       <c r="D61" t="n">
-        <v>100000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Mayfair Community Development Corporation</t>
+          <t>Mt. Airy U.S.A.</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C62" t="n">
         <v>2013</v>
@@ -27156,14 +27152,14 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Mt. Airy U.S.A.</t>
+          <t>New Kensington Community Development Corporation</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C63" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="D63" t="n">
         <v>85000</v>
@@ -27172,78 +27168,78 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>New Kensington Community Development Corporation</t>
+          <t>Nicetown Community Development Corporation</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C64" t="n">
-        <v>2012</v>
+        <v>2009</v>
       </c>
       <c r="D64" t="n">
-        <v>85000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Nicetown Community Development Corporation</t>
+          <t>Nueva Esperanza Inc.</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C65" t="n">
-        <v>2019</v>
+        <v>2013</v>
       </c>
       <c r="D65" t="n">
-        <v>100000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Nueva Esperanza, Inc.</t>
+          <t>Ogontz Ave Revitalization Corporation</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C66" t="n">
-        <v>2013</v>
+        <v>2009</v>
       </c>
       <c r="D66" t="n">
-        <v>85000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Old City Community Fund</t>
+          <t>People's Emergency Center CDC</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C67" t="n">
-        <v>2017</v>
+        <v>2012</v>
       </c>
       <c r="D67" t="n">
-        <v>100</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>People’s Emergency Center CDC</t>
+          <t>Philabundance</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C68" t="n">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="D68" t="n">
         <v>85000</v>
@@ -27252,14 +27248,14 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Philabundance, HFI</t>
+          <t>Philadelphia Association of Community Development Corporations</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C69" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="D69" t="n">
         <v>85000</v>
@@ -27268,14 +27264,14 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Philadelphia Association of Community Development Corporations, NPI</t>
+          <t>Philadelphia Chinatown Development Corporation</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C70" t="n">
-        <v>2012</v>
+        <v>2014</v>
       </c>
       <c r="D70" t="n">
         <v>85000</v>
@@ -27284,14 +27280,14 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Philadelphia Chinatown Development Corporation</t>
+          <t>Philadelphia Local Initiatives Support Corporation</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C71" t="n">
-        <v>2014</v>
+        <v>2012</v>
       </c>
       <c r="D71" t="n">
         <v>85000</v>
@@ -27300,14 +27296,14 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Philadelphia Local Initiatives Support Corporation, NPI</t>
+          <t>Project H.O.M.E.</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C72" t="n">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="D72" t="n">
         <v>85000</v>
@@ -27316,14 +27312,14 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Project H.O.M.E.</t>
+          <t>Regional Housing Legal Services</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C73" t="n">
-        <v>2013</v>
+        <v>2014</v>
       </c>
       <c r="D73" t="n">
         <v>85000</v>
@@ -27332,30 +27328,30 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Regional Housing Legal Services-NPI (business sponsor dropped out 2018)</t>
+          <t>Roxborough Development Corporation</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C74" t="n">
-        <v>2014</v>
+        <v>2012</v>
       </c>
       <c r="D74" t="n">
-        <v>0</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Roxborough Development Corporation</t>
+          <t>Schuylkill River Development Corporation</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C75" t="n">
-        <v>2012</v>
+        <v>2014</v>
       </c>
       <c r="D75" t="n">
         <v>85000</v>
@@ -27364,62 +27360,62 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Schuylkill River Development Corporation (SRDC)</t>
+          <t>South of South Neighborhood Association</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C76" t="n">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="D76" t="n">
-        <v>85000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>SEAMAAC, Inc.</t>
+          <t>Southwest Community Development Corporation</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C77" t="n">
-        <v>2019</v>
+        <v>2012</v>
       </c>
       <c r="D77" t="n">
-        <v>100000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>South of South Neighborhood Association</t>
+          <t>Spring Garden Community Development Corporation</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C78" t="n">
-        <v>2015</v>
+        <v>2013</v>
       </c>
       <c r="D78" t="n">
-        <v>100000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Southwest Community Development Corporation</t>
+          <t>Tacony Community Development Corporation</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C79" t="n">
-        <v>2012</v>
+        <v>2014</v>
       </c>
       <c r="D79" t="n">
         <v>85000</v>
@@ -27428,14 +27424,14 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Spring Garden Community Development Corporation</t>
+          <t>The Allegheny West Foundation</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C80" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="D80" t="n">
         <v>85000</v>
@@ -27444,33 +27440,33 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Tacony Community Development Corporation</t>
+          <t>The Enterprise Center Community Development Corporation</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C81" t="n">
-        <v>2014</v>
+        <v>2009</v>
       </c>
       <c r="D81" t="n">
-        <v>85000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>The Allegheny West Foundation</t>
+          <t>The Partnership Community Development Corporation</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C82" t="n">
-        <v>2019</v>
+        <v>2013</v>
       </c>
       <c r="D82" t="n">
-        <v>100000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="83">
@@ -27480,7 +27476,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C83" t="n">
         <v>2013</v>
@@ -27496,7 +27492,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C84" t="n">
         <v>2015</v>
@@ -27512,7 +27508,7 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="C85" t="n">
         <v>2010</v>
@@ -27528,7 +27524,7 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C86" t="n">
         <v>2012</v>
@@ -27540,11 +27536,11 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Asociaciόn Puertorriqueños En Marcha, Inc</t>
+          <t>Asociación Puertorriqueños En Marcha Inc</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C87" t="n">
         <v>2015</v>
@@ -27556,11 +27552,11 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Beech Interplex, Inc.</t>
+          <t>Beech Interplex Inc.</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C88" t="n">
         <v>2013</v>
@@ -27576,7 +27572,7 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C89" t="n">
         <v>2012</v>
@@ -27592,7 +27588,7 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C90" t="n">
         <v>2013</v>
@@ -27604,11 +27600,11 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Common Market Philadelphia, Inc., HFI</t>
+          <t>Common Market Philadelphia Inc.</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C91" t="n">
         <v>2013</v>
@@ -27620,11 +27616,11 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Community Design Collaborative, NPI</t>
+          <t>Community Design Collaborative</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C92" t="n">
         <v>2012</v>
@@ -27636,11 +27632,11 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Delaware River City Corporation (DRCC)</t>
+          <t>Delaware River City Corporation</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C93" t="n">
         <v>2017</v>
@@ -27656,7 +27652,7 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C94" t="n">
         <v>2013</v>
@@ -27672,7 +27668,7 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C95" t="n">
         <v>2012</v>
@@ -27688,7 +27684,7 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C96" t="n">
         <v>2013</v>
@@ -27704,7 +27700,7 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C97" t="n">
         <v>2014</v>
@@ -27720,7 +27716,7 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C98" t="n">
         <v>2015</v>
@@ -27736,7 +27732,7 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C99" t="n">
         <v>2012</v>
@@ -27748,30 +27744,30 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Germantown United Community Development Corporation</t>
+          <t>HACE aka Hispanic Assoc. of Contractors &amp; Enterprises</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C100" t="n">
-        <v>2019</v>
+        <v>2013</v>
       </c>
       <c r="D100" t="n">
-        <v>100000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>HACE aka Hispanic Assoc. of Contractors &amp; Enterprises</t>
+          <t>Impact Services Corporation</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C101" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="D101" t="n">
         <v>85000</v>
@@ -27780,33 +27776,33 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Impact Services Corporation</t>
+          <t>Manayunk Development Corporation</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C102" t="n">
-        <v>2012</v>
+        <v>2010</v>
       </c>
       <c r="D102" t="n">
-        <v>85000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Mayfair Business Improvement District (BID)</t>
+          <t>Mayfair Community Development Corporation</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C103" t="n">
-        <v>2020</v>
+        <v>2013</v>
       </c>
       <c r="D103" t="n">
-        <v>100000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="104">
@@ -27816,7 +27812,7 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C104" t="n">
         <v>2013</v>
@@ -27832,7 +27828,7 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C105" t="n">
         <v>2012</v>
@@ -27844,14 +27840,14 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>New Manayunk Corporation</t>
+          <t>Nicetown Community Development Corporation</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C106" t="n">
-        <v>2020</v>
+        <v>2009</v>
       </c>
       <c r="D106" t="n">
         <v>100000</v>
@@ -27860,33 +27856,33 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Nicetown Community Development Corporation</t>
+          <t>Nueva Esperanza Inc.</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C107" t="n">
-        <v>2019</v>
+        <v>2013</v>
       </c>
       <c r="D107" t="n">
-        <v>100000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Nueva Esperanza, Inc.</t>
+          <t>Ogontz Ave Revitalization Corporation</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C108" t="n">
-        <v>2013</v>
+        <v>2009</v>
       </c>
       <c r="D108" t="n">
-        <v>85000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="109">
@@ -27896,23 +27892,23 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C109" t="n">
         <v>2017</v>
       </c>
       <c r="D109" t="n">
-        <v>100</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>People’s Emergency Center CDC</t>
+          <t>People's Emergency Center CDC</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C110" t="n">
         <v>2012</v>
@@ -27924,11 +27920,11 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Philabundance, HFI</t>
+          <t>Philabundance</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C111" t="n">
         <v>2013</v>
@@ -27940,11 +27936,11 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Philadelphia Association of Community Development Corporations, NPI</t>
+          <t>Philadelphia Association of Community Development Corporations</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C112" t="n">
         <v>2012</v>
@@ -27960,7 +27956,7 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C113" t="n">
         <v>2014</v>
@@ -27972,11 +27968,11 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Philadelphia Local Initiatives Support Corporation, NPI</t>
+          <t>Philadelphia Local Initiatives Support Corporation</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C114" t="n">
         <v>2012</v>
@@ -27992,7 +27988,7 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C115" t="n">
         <v>2013</v>
@@ -28004,14 +28000,14 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Roxborough Development Corporation</t>
+          <t>Regional Housing Legal Services</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C116" t="n">
-        <v>2012</v>
+        <v>2014</v>
       </c>
       <c r="D116" t="n">
         <v>85000</v>
@@ -28020,14 +28016,14 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Schuylkill River Development Corporation (SRDC)</t>
+          <t>Roxborough Development Corporation</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C117" t="n">
-        <v>2014</v>
+        <v>2012</v>
       </c>
       <c r="D117" t="n">
         <v>85000</v>
@@ -28036,17 +28032,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>SEAMAAC, Inc.</t>
+          <t>Schuylkill River Development Corporation</t>
         </is>
       </c>
       <c r="B118" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C118" t="n">
-        <v>2019</v>
+        <v>2014</v>
       </c>
       <c r="D118" t="n">
-        <v>100000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="119">
@@ -28056,7 +28052,7 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C119" t="n">
         <v>2015</v>
@@ -28068,30 +28064,30 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>South Street Headhouse District Foundation</t>
+          <t>Southwest Community Development Corporation</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C120" t="n">
-        <v>2020</v>
+        <v>2012</v>
       </c>
       <c r="D120" t="n">
-        <v>100000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Southwest Community Development Corporation</t>
+          <t>Spring Garden Community Development Corporation</t>
         </is>
       </c>
       <c r="B121" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C121" t="n">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="D121" t="n">
         <v>85000</v>
@@ -28100,14 +28096,14 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Spring Garden Community Development Corporation</t>
+          <t>Tacony Community Development Corporation</t>
         </is>
       </c>
       <c r="B122" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C122" t="n">
-        <v>2013</v>
+        <v>2014</v>
       </c>
       <c r="D122" t="n">
         <v>85000</v>
@@ -28116,14 +28112,14 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Tacony Community Development Corporation</t>
+          <t>The Allegheny West Foundation</t>
         </is>
       </c>
       <c r="B123" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C123" t="n">
-        <v>2014</v>
+        <v>2012</v>
       </c>
       <c r="D123" t="n">
         <v>85000</v>
@@ -28132,14 +28128,14 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>The Allegheny West Foundation</t>
+          <t>The Enterprise Center Community Development Corporation</t>
         </is>
       </c>
       <c r="B124" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C124" t="n">
-        <v>2019</v>
+        <v>2009</v>
       </c>
       <c r="D124" t="n">
         <v>100000</v>
@@ -28148,48 +28144,2048 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>The Enterprise Center CDC</t>
+          <t>The Village of Arts and Humanities</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C125" t="n">
-        <v>2020</v>
+        <v>2013</v>
       </c>
       <c r="D125" t="n">
-        <v>100000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>The Village of Arts and Humanities</t>
+          <t>University City District</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="C126" t="n">
-        <v>2013</v>
+        <v>2015</v>
       </c>
       <c r="D126" t="n">
-        <v>85000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
+          <t>Wynnefield Overbrook Revitalization Corp.</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>2017</v>
+      </c>
+      <c r="C127" t="n">
+        <v>2010</v>
+      </c>
+      <c r="D127" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>ACHIEVEability</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C128" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D128" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Asociación Puertorriqueños En Marcha Inc</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C129" t="n">
+        <v>2015</v>
+      </c>
+      <c r="D129" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Beech Interplex Inc.</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C130" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D130" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Central Philadelphia Development Corporation</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C131" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D131" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Chestnut Hill Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C132" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D132" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Common Market Philadelphia Inc.</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C133" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D133" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Community Design Collaborative</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C134" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D134" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Delaware River City Corporation</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C135" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D135" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Delaware River Waterfront Corporation</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C136" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D136" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>East Falls Development Corporation</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C137" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D137" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>East Passyunk Avenue Improvement District</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C138" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D138" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Fairmount Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C139" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D139" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Francisville Neighborhood Development Corporation</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C140" t="n">
+        <v>2015</v>
+      </c>
+      <c r="D140" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Frankford Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C141" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D141" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>HACE aka Hispanic Assoc. of Contractors &amp; Enterprises</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C142" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D142" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Impact Services Corporation</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C143" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D143" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Manayunk Development Corporation</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C144" t="n">
+        <v>2010</v>
+      </c>
+      <c r="D144" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Mayfair Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C145" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D145" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Mt. Airy U.S.A.</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C146" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D146" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>New Kensington Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C147" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D147" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Nicetown Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C148" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D148" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Nueva Esperanza Inc.</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C149" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D149" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Ogontz Ave Revitalization Corporation</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C150" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D150" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Old City Community Fund</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C151" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D151" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>People's Emergency Center CDC</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C152" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D152" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Philabundance</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C153" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D153" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Philadelphia Association of Community Development Corporations</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C154" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D154" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Philadelphia Chinatown Development Corporation</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C155" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D155" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Philadelphia Local Initiatives Support Corporation</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C156" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D156" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Project H.O.M.E.</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C157" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D157" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Regional Housing Legal Services</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C158" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D158" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Roxborough Development Corporation</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C159" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D159" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Schuylkill River Development Corporation</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C160" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D160" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>South of South Neighborhood Association</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C161" t="n">
+        <v>2015</v>
+      </c>
+      <c r="D161" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Southwest Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C162" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D162" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Spring Garden Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C163" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D163" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Tacony Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C164" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D164" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>The Enterprise Center Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C165" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D165" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>The Village of Arts and Humanities</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C166" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D166" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
           <t>University City District</t>
         </is>
       </c>
-      <c r="B127" t="n">
+      <c r="B167" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C167" t="n">
+        <v>2015</v>
+      </c>
+      <c r="D167" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Wynnefield Overbrook Revitalization Corp.</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>2018</v>
+      </c>
+      <c r="C168" t="n">
+        <v>2010</v>
+      </c>
+      <c r="D168" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>ACHIEVEability</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C169" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D169" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Asociaciόn Puertorriqueños En Marcha, Inc</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C170" t="n">
+        <v>2015</v>
+      </c>
+      <c r="D170" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Beech Interplex, Inc.</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C171" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D171" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Central Philadelphia Development Corporation</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C172" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D172" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Chestnut Hill Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C173" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D173" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Common Market Philadelphia, Inc., HFI</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C174" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D174" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Community Design Collaborative, NPI</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C175" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D175" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Delaware River City Corporation (DRCC)</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C176" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D176" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Delaware River Waterfront Corporation</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C177" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D177" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>East Falls Development Corporation</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C178" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D178" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>East Passyunk Avenue Improvement District</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C179" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D179" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Fairmount Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C180" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D180" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Francisville Neighborhood Development Corporation</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C181" t="n">
+        <v>2015</v>
+      </c>
+      <c r="D181" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Frankford Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C182" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D182" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Germantown United Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C183" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D183" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>HACE aka Hispanic Assoc. of Contractors &amp; Enterprises</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C184" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D184" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Impact Services Corporation</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C185" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D185" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Manayunk Development Corporation</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C186" t="n">
+        <v>2010</v>
+      </c>
+      <c r="D186" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Mayfair Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C187" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D187" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Mt. Airy U.S.A.</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C188" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D188" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>New Kensington Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C189" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D189" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Nicetown Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C190" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D190" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Nueva Esperanza, Inc.</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C191" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D191" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Old City Community Fund</t>
+        </is>
+      </c>
+      <c r="B192" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C192" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D192" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>People’s Emergency Center CDC</t>
+        </is>
+      </c>
+      <c r="B193" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C193" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D193" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Philabundance, HFI</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C194" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D194" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Philadelphia Association of Community Development Corporations, NPI</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C195" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D195" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Philadelphia Chinatown Development Corporation</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C196" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D196" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Philadelphia Local Initiatives Support Corporation, NPI</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C197" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D197" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Project H.O.M.E.</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C198" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D198" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Regional Housing Legal Services-NPI (business sponsor dropped out 2018)</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C199" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D199" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Roxborough Development Corporation</t>
+        </is>
+      </c>
+      <c r="B200" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C200" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D200" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Schuylkill River Development Corporation (SRDC)</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C201" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D201" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>SEAMAAC, Inc.</t>
+        </is>
+      </c>
+      <c r="B202" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C202" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D202" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>South of South Neighborhood Association</t>
+        </is>
+      </c>
+      <c r="B203" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C203" t="n">
+        <v>2015</v>
+      </c>
+      <c r="D203" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Southwest Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B204" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C204" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D204" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Spring Garden Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C205" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D205" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Tacony Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C206" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D206" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>The Allegheny West Foundation</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C207" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D207" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>The Village of Arts and Humanities</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C208" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D208" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>University City District</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C209" t="n">
+        <v>2015</v>
+      </c>
+      <c r="D209" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Wynnefield Overbrook Revitalization Corp.</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>2019</v>
+      </c>
+      <c r="C210" t="n">
+        <v>2010</v>
+      </c>
+      <c r="D210" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>ACHIEVEability</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
         <v>2020</v>
       </c>
-      <c r="C127" t="n">
+      <c r="C211" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D211" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Asociaciόn Puertorriqueños En Marcha, Inc</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C212" t="n">
         <v>2015</v>
       </c>
-      <c r="D127" t="n">
+      <c r="D212" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Beech Interplex, Inc.</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C213" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D213" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Central Philadelphia Development Corporation</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C214" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D214" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Chestnut Hill Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C215" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D215" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Common Market Philadelphia, Inc., HFI</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C216" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D216" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Community Design Collaborative, NPI</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C217" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D217" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Delaware River City Corporation (DRCC)</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C218" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D218" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Delaware River Waterfront Corporation</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C219" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D219" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>East Falls Development Corporation</t>
+        </is>
+      </c>
+      <c r="B220" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C220" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D220" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>East Passyunk Avenue Improvement District</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C221" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D221" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Fairmount Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C222" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D222" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Francisville Neighborhood Development Corporation</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C223" t="n">
+        <v>2015</v>
+      </c>
+      <c r="D223" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Frankford Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B224" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C224" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D224" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Germantown United Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B225" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C225" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D225" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>HACE aka Hispanic Assoc. of Contractors &amp; Enterprises</t>
+        </is>
+      </c>
+      <c r="B226" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C226" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D226" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Impact Services Corporation</t>
+        </is>
+      </c>
+      <c r="B227" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C227" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D227" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Mayfair Business Improvement District (BID)</t>
+        </is>
+      </c>
+      <c r="B228" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C228" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D228" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Mt. Airy U.S.A.</t>
+        </is>
+      </c>
+      <c r="B229" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C229" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D229" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>New Kensington Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B230" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C230" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D230" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>New Manayunk Corporation</t>
+        </is>
+      </c>
+      <c r="B231" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C231" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D231" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Nicetown Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B232" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C232" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D232" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Nueva Esperanza, Inc.</t>
+        </is>
+      </c>
+      <c r="B233" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C233" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D233" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Old City Community Fund</t>
+        </is>
+      </c>
+      <c r="B234" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C234" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D234" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>People’s Emergency Center CDC</t>
+        </is>
+      </c>
+      <c r="B235" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C235" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D235" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Philabundance, HFI</t>
+        </is>
+      </c>
+      <c r="B236" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C236" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D236" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Philadelphia Association of Community Development Corporations, NPI</t>
+        </is>
+      </c>
+      <c r="B237" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C237" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D237" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Philadelphia Chinatown Development Corporation</t>
+        </is>
+      </c>
+      <c r="B238" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C238" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D238" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Philadelphia Local Initiatives Support Corporation, NPI</t>
+        </is>
+      </c>
+      <c r="B239" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C239" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D239" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Project H.O.M.E.</t>
+        </is>
+      </c>
+      <c r="B240" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C240" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D240" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Roxborough Development Corporation</t>
+        </is>
+      </c>
+      <c r="B241" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C241" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D241" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Schuylkill River Development Corporation (SRDC)</t>
+        </is>
+      </c>
+      <c r="B242" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C242" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D242" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>SEAMAAC, Inc.</t>
+        </is>
+      </c>
+      <c r="B243" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C243" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D243" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>South of South Neighborhood Association</t>
+        </is>
+      </c>
+      <c r="B244" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C244" t="n">
+        <v>2015</v>
+      </c>
+      <c r="D244" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>South Street Headhouse District Foundation</t>
+        </is>
+      </c>
+      <c r="B245" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C245" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D245" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Southwest Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B246" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C246" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D246" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Spring Garden Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B247" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C247" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D247" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Tacony Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B248" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C248" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D248" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>The Allegheny West Foundation</t>
+        </is>
+      </c>
+      <c r="B249" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C249" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D249" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>The Enterprise Center CDC</t>
+        </is>
+      </c>
+      <c r="B250" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C250" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D250" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>The Village of Arts and Humanities</t>
+        </is>
+      </c>
+      <c r="B251" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C251" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D251" t="n">
+        <v>85000</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>University City District</t>
+        </is>
+      </c>
+      <c r="B252" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C252" t="n">
+        <v>2015</v>
+      </c>
+      <c r="D252" t="n">
         <v>100000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: dedicated Temple Archives sheet tab, per Ben's ask
Ben wanted the Temple-archives CDC finds broken out into their own
sheet tab rather than folded into Roster. Added a "Temple Archives"
tab (organization, which finding aid it came from, EIN match status,
years filed, executive, news/Inquirer counts, notes) so it's a
standalone review surface instead of scattered rows in the main
roster. Also threads the source collection through to the org detail
page's archive callout on the web app.
</commit_message>
<xml_diff>
--- a/output/corridor_dataset.xlsx
+++ b/output/corridor_dataset.xlsx
@@ -8,13 +8,14 @@
   </bookViews>
   <sheets>
     <sheet name="Roster" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Leadership" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Financial History" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Tax Credit" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="990 PDFs" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="News &amp; Sources" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Signals" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="About" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Temple Archives" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Leadership" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Financial History" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Tax Credit" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="990 PDFs" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="News &amp; Sources" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Signals" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="About" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -41,7 +42,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -65,6 +66,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F6D6D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00EAF1FE"/>
       </patternFill>
     </fill>
@@ -81,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -89,6 +95,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5165,6 +5172,1151 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="70" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Organization</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Archive collection</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>EIN</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Match status</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Years filed</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Executive director</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>News articles found</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Inquirer articles</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Advocate Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PACDC Records (SCRC 241)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>231706238</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>PACDC member CDC, active 2000-2004 per PACDC's own records (Temple University Special Collections Research Center).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Brewerytown CDC</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PACDC Records (SCRC 241)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>473603645</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>PACDC member CDC, active as of 2006 per Temple University Special Collections Research Center PACDC records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Calvary CDC</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PACDC Records (SCRC 241)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>883037723</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>PACDC yearbook member CDC, per Temple University Special Collections Research Center PACDC records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Central Germantown Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Germantown Settlement Records (KER0314221)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>232888616</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Predecessor/counterpart to Greater Germantown Housing Development Corporation; own minutes and inter-org agreements survive through at least 1988.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>East of Broad Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Kensington Action Now Records (Acc 705)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>needs manual lookup</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Named in the Kensington Action Now records at Temple's Special Collections Research Center.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Faith CDC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PACDC Records (SCRC 241)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>43673651</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>13</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Mehboob Khan</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>PACDC yearbook member CDC, per Temple University Special Collections Research Center PACDC records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>First Baptist Church of Paschall Development Corporation</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Germantown Settlement Records (KER0314221)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>231365253</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Faith-based CDC; filed a statement of need with Greater Germantown Housing Development Corporation, 1990.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Frankford United Neighbors CDC</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PACDC Records (SCRC 241)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>237217565</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>PACDC yearbook member CDC, per Temple University Special Collections Research Center PACDC records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Germantown Settlement</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Germantown Settlement Records (KER0314221)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>needs manual lookup</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="n">
+        <v>8</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Founded 1934 from the merger of Morton Street Day Nursery (est. 1884) and Germantown Community Center (est. 1920). Grew into one of Philadelphia's largest CDCs before financial and governance troubles led to its collapse and dissolution in the 2000s. 455-page records collection at Temple, the largest in this find.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Greater Germantown Housing Development Corporation</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Germantown Settlement Records (KER0314221)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>232024975</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>7</v>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Active by 1976, succeeding Central Germantown Community Development Corporation; ran housing rehab and homeowner technical-assistance programs into the early 1990s. 455-page records collection at Temple's Special Collections Research Center.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Hawthorne Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PACDC Records (SCRC 241)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>needs manual lookup</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Wrote a neighborhood plan in 1995, per Temple University Special Collections Research Center PACDC records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Hunting Park Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PACDC Records (SCRC 241)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>264300365</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>13</v>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>PACDC yearbook member CDC, per Temple University Special Collections Research Center PACDC records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Jefferson Manor Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PACDC Records (SCRC 241)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>needs manual lookup</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>PACDC yearbook member CDC, per Temple University Special Collections Research Center PACDC records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Kensington Area Revitalization Project</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Kensington Action Now Records (Acc 705)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>844037072</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Marc D Collazzo</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Spun out of the Kensington Action Now coalition on 1980-05-09 to acquire, renovate, and sell abandoned properties.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Logan Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Regional Council of Neighborhood Organizations Records (Acc 658 et al.)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>872025770</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="n">
+        <v>7</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Named in the Regional Council of Neighborhood Organizations (RCNO) records, 1986.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Mt. Airy Village Development Corporation</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PACDC Records (SCRC 241)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>260898815</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>12</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Isaac Ewell</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>PACDC yearbook member CDC, per Temple University Special Collections Research Center PACDC records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Olde Kensington Redevelopment Corporation</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Olde Kensington Senior Housing Associates Records (JL0503221)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>834158522</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>John Williams</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Chartered 1968 to develop low-cost housing in Kensington. Formed O.K. Improvement Inc. (1979) and Olde Kensington Senior Housing Associates (1982), which built Sylvia Barg Plaza (opened 1986) and dissolved after selling the building in 2014.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>People's Emergency Center CDC</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PACDC Records (SCRC 241)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>needs manual lookup</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="n">
+        <v>2</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>PACDC member CDC with retail-analysis and general records, 2002-2007, per Temple University Special Collections Research Center PACDC records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Roxborough Development Corporation</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PACDC Records (SCRC 241)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>232705347</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>12</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Jax Cusack</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>8</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>PACDC member CDC, active as of 2005 per Temple University Special Collections Research Center PACDC records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sheridan Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>PACDC Records (SCRC 241)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>needs manual lookup</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>PACDC yearbook member CDC, per Temple University Special Collections Research Center PACDC records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Socca Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PACDC Records (SCRC 241)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>needs manual lookup</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>PACDC correspondent (contact: Patricia Evans), 1994; no further detail found in the archives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>South Philadelphia Community Development Corporation</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>West Philadelphia Corporation Records (Acc 350 et al.)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>991321510</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Named in the West Philadelphia Corporation records, active 1967-1969; likely long dissolved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Southwest Germantown CDC</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Regional Council of Neighborhood Organizations Records (Acc 658 et al.)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>needs manual lookup</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Named in the Regional Council of Neighborhood Organizations (RCNO) records, 1986.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Sunrise CDC</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>PACDC Records (SCRC 241)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>932447863</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>PACDC member CDC, active as of 2006 per Temple University Special Collections Research Center PACDC records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Tenth Memorial Non-Profit Development Corporation</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>PACDC Records (SCRC 241)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>222538855</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>13</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Rev William B Moore</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Faith-based CDC tied to Tenth Memorial Baptist Church; PACDC correspondence lists it as a non-member org, 1993-1994.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Weccacoe Development Association</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Weccacoe Development Association Records (Acc 932)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>222646975</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Founded 1985 to build and rehab low- and moderate-income housing and clear vacant properties in the Weccacoe (Queen Village/Bella Vista) area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>West Oak Lane CDC</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>PACDC Records (SCRC 241)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>232142704</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>11</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Donald T Stafford</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>PACDC member CDC; wrote a neighborhood commercial-corridor plan in 1995, per Temple University Special Collections Research Center PACDC records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>West Philadelphia Economic Development Corporation</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>PACDC Records (SCRC 241)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>844201970</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Named in PACDC's 1994 records; distinct from West Philadelphia Partnership/Partnership CDC, no further detail found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Yorktown CDC</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>PACDC Records (SCRC 241)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>232642355</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>12</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Renee V Drayton</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>PACDC member CDC, active as of 2006 per Temple University Special Collections Research Center PACDC records.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F496"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5209,30 +6361,30 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>African Cultural Alliance of North America</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>233062024</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Voffee Jabateh</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="E2" s="5" t="n">
         <v>122646</v>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -5447,30 +6599,30 @@
       <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Arab-American CDC</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>311620684</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Asif Hussein</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>President</t>
         </is>
       </c>
-      <c r="E11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="E11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -5529,30 +6681,30 @@
       <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Asociación Puertorriqueños en Marcha (APM)</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>231930630</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Nilda I Ruiz</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>President/Ceo</t>
         </is>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E14" s="5" t="n">
         <v>350774</v>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -5793,30 +6945,30 @@
       <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Beech Interplex</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>521693162</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Kenneth Scott</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>President Ce</t>
         </is>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="E24" s="5" t="n">
         <v>120000</v>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -5953,30 +7105,30 @@
       <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>Called To Serve CDC</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>464404323</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>Michael Major</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>President</t>
         </is>
       </c>
-      <c r="E30" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="E30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -6087,30 +7239,30 @@
       <c r="F34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>Centennial Parkside CDC</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>474815728</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>Jessi Ray Koch</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D35" s="5" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="E35" s="4" t="n">
+      <c r="E35" s="5" t="n">
         <v>77289</v>
       </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="F35" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -6377,30 +7529,30 @@
       <c r="F45" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+      <c r="A46" s="5" t="inlineStr">
         <is>
           <t>Chestnut Hill CDC</t>
         </is>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B46" s="5" t="inlineStr">
         <is>
           <t>274673757</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C46" s="5" t="inlineStr">
         <is>
           <t>Richard Snowden</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D46" s="5" t="inlineStr">
         <is>
           <t>President</t>
         </is>
       </c>
-      <c r="E46" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
+      <c r="E46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -6485,30 +7637,30 @@
       <c r="F49" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+      <c r="A50" s="5" t="inlineStr">
         <is>
           <t>Community of Compassion CDC</t>
         </is>
       </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>331035662</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C50" s="5" t="inlineStr">
         <is>
           <t>W Lonnie Herndon</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
+      <c r="D50" s="5" t="inlineStr">
         <is>
           <t>President</t>
         </is>
       </c>
-      <c r="E50" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F50" s="4" t="inlineStr">
+      <c r="E50" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -6723,30 +7875,30 @@
       <c r="F58" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="inlineStr">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>Community Ventures</t>
         </is>
       </c>
-      <c r="B59" s="4" t="inlineStr">
+      <c r="B59" s="5" t="inlineStr">
         <is>
           <t>232462126</t>
         </is>
       </c>
-      <c r="C59" s="4" t="inlineStr">
+      <c r="C59" s="5" t="inlineStr">
         <is>
           <t>David Lafontaine</t>
         </is>
       </c>
-      <c r="D59" s="4" t="inlineStr">
+      <c r="D59" s="5" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="E59" s="4" t="n">
+      <c r="E59" s="5" t="n">
         <v>131284</v>
       </c>
-      <c r="F59" s="4" t="inlineStr">
+      <c r="F59" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -6987,30 +8139,30 @@
       <c r="F68" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="4" t="inlineStr">
+      <c r="A69" s="5" t="inlineStr">
         <is>
           <t>East Falls Development Corporation</t>
         </is>
       </c>
-      <c r="B69" s="4" t="inlineStr">
+      <c r="B69" s="5" t="inlineStr">
         <is>
           <t>232805925</t>
         </is>
       </c>
-      <c r="C69" s="4" t="inlineStr">
+      <c r="C69" s="5" t="inlineStr">
         <is>
           <t>Michelle Feldman</t>
         </is>
       </c>
-      <c r="D69" s="4" t="inlineStr">
+      <c r="D69" s="5" t="inlineStr">
         <is>
           <t>Exec Director</t>
         </is>
       </c>
-      <c r="E69" s="4" t="n">
+      <c r="E69" s="5" t="n">
         <v>77449</v>
       </c>
-      <c r="F69" s="4" t="inlineStr">
+      <c r="F69" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -7251,60 +8403,60 @@
       <c r="F78" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="4" t="inlineStr">
+      <c r="A79" s="5" t="inlineStr">
         <is>
           <t>Empowered CDC</t>
         </is>
       </c>
-      <c r="B79" s="4" t="inlineStr">
+      <c r="B79" s="5" t="inlineStr">
         <is>
           <t>845037676</t>
         </is>
       </c>
-      <c r="C79" s="4" t="inlineStr">
+      <c r="C79" s="5" t="inlineStr">
         <is>
           <t>Xeyah T Martin</t>
         </is>
       </c>
-      <c r="D79" s="4" t="inlineStr">
+      <c r="D79" s="5" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="E79" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F79" s="4" t="inlineStr">
+      <c r="E79" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="4" t="inlineStr">
+      <c r="A80" s="5" t="inlineStr">
         <is>
           <t>Esperanza</t>
         </is>
       </c>
-      <c r="B80" s="4" t="inlineStr">
+      <c r="B80" s="5" t="inlineStr">
         <is>
           <t>232552707</t>
         </is>
       </c>
-      <c r="C80" s="4" t="inlineStr">
+      <c r="C80" s="5" t="inlineStr">
         <is>
           <t>Reverend Luis Cortes Jr</t>
         </is>
       </c>
-      <c r="D80" s="4" t="inlineStr">
+      <c r="D80" s="5" t="inlineStr">
         <is>
           <t>President &amp; Ceo</t>
         </is>
       </c>
-      <c r="E80" s="4" t="n">
+      <c r="E80" s="5" t="n">
         <v>396023</v>
       </c>
-      <c r="F80" s="4" t="inlineStr">
+      <c r="F80" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -7545,30 +8697,30 @@
       <c r="F89" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="4" t="inlineStr">
+      <c r="A90" s="5" t="inlineStr">
         <is>
           <t>Frankford CDC</t>
         </is>
       </c>
-      <c r="B90" s="4" t="inlineStr">
+      <c r="B90" s="5" t="inlineStr">
         <is>
           <t>232738932</t>
         </is>
       </c>
-      <c r="C90" s="4" t="inlineStr">
+      <c r="C90" s="5" t="inlineStr">
         <is>
           <t>Kimberly Washington</t>
         </is>
       </c>
-      <c r="D90" s="4" t="inlineStr">
+      <c r="D90" s="5" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="E90" s="4" t="n">
+      <c r="E90" s="5" t="n">
         <v>123654</v>
       </c>
-      <c r="F90" s="4" t="inlineStr">
+      <c r="F90" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -7809,30 +8961,30 @@
       <c r="F99" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="A100" s="4" t="inlineStr">
+      <c r="A100" s="5" t="inlineStr">
         <is>
           <t>Germantown United CDC</t>
         </is>
       </c>
-      <c r="B100" s="4" t="inlineStr">
+      <c r="B100" s="5" t="inlineStr">
         <is>
           <t>453739378</t>
         </is>
       </c>
-      <c r="C100" s="4" t="inlineStr">
+      <c r="C100" s="5" t="inlineStr">
         <is>
           <t>Emaleigh Doley</t>
         </is>
       </c>
-      <c r="D100" s="4" t="inlineStr">
+      <c r="D100" s="5" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="E100" s="4" t="n">
+      <c r="E100" s="5" t="n">
         <v>44000</v>
       </c>
-      <c r="F100" s="4" t="inlineStr">
+      <c r="F100" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -8073,30 +9225,30 @@
       <c r="F109" t="inlineStr"/>
     </row>
     <row r="110">
-      <c r="A110" s="4" t="inlineStr">
+      <c r="A110" s="5" t="inlineStr">
         <is>
           <t>Habitat for Humanity Philadelphia</t>
         </is>
       </c>
-      <c r="B110" s="4" t="inlineStr">
+      <c r="B110" s="5" t="inlineStr">
         <is>
           <t>421580163</t>
         </is>
       </c>
-      <c r="C110" s="4" t="inlineStr">
+      <c r="C110" s="5" t="inlineStr">
         <is>
           <t>Corinne O'connell</t>
         </is>
       </c>
-      <c r="D110" s="4" t="inlineStr">
+      <c r="D110" s="5" t="inlineStr">
         <is>
           <t>Chief Executive Officer</t>
         </is>
       </c>
-      <c r="E110" s="4" t="n">
+      <c r="E110" s="5" t="n">
         <v>226043</v>
       </c>
-      <c r="F110" s="4" t="inlineStr">
+      <c r="F110" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -8337,30 +9489,30 @@
       <c r="F119" t="inlineStr"/>
     </row>
     <row r="120">
-      <c r="A120" s="4" t="inlineStr">
+      <c r="A120" s="5" t="inlineStr">
         <is>
           <t>HopePHL</t>
         </is>
       </c>
-      <c r="B120" s="4" t="inlineStr">
+      <c r="B120" s="5" t="inlineStr">
         <is>
           <t>232017882</t>
         </is>
       </c>
-      <c r="C120" s="4" t="inlineStr">
+      <c r="C120" s="5" t="inlineStr">
         <is>
           <t>Kathleen Desmond</t>
         </is>
       </c>
-      <c r="D120" s="4" t="inlineStr">
+      <c r="D120" s="5" t="inlineStr">
         <is>
           <t>President</t>
         </is>
       </c>
-      <c r="E120" s="4" t="n">
+      <c r="E120" s="5" t="n">
         <v>176533</v>
       </c>
-      <c r="F120" s="4" t="inlineStr">
+      <c r="F120" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -8861,30 +10013,30 @@
       <c r="F139" t="inlineStr"/>
     </row>
     <row r="140">
-      <c r="A140" s="4" t="inlineStr">
+      <c r="A140" s="5" t="inlineStr">
         <is>
           <t>Impact Services Corporation</t>
         </is>
       </c>
-      <c r="B140" s="4" t="inlineStr">
+      <c r="B140" s="5" t="inlineStr">
         <is>
           <t>232087348</t>
         </is>
       </c>
-      <c r="C140" s="4" t="inlineStr">
+      <c r="C140" s="5" t="inlineStr">
         <is>
           <t>Casey O'donnell</t>
         </is>
       </c>
-      <c r="D140" s="4" t="inlineStr">
+      <c r="D140" s="5" t="inlineStr">
         <is>
           <t>President &amp; Ceo</t>
         </is>
       </c>
-      <c r="E140" s="4" t="n">
+      <c r="E140" s="5" t="n">
         <v>248675</v>
       </c>
-      <c r="F140" s="4" t="inlineStr">
+      <c r="F140" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -9125,30 +10277,30 @@
       <c r="F149" t="inlineStr"/>
     </row>
     <row r="150">
-      <c r="A150" s="4" t="inlineStr">
+      <c r="A150" s="5" t="inlineStr">
         <is>
           <t>Inglis Housing Corporation</t>
         </is>
       </c>
-      <c r="B150" s="4" t="inlineStr">
+      <c r="B150" s="5" t="inlineStr">
         <is>
           <t>232326550</t>
         </is>
       </c>
-      <c r="C150" s="4" t="inlineStr">
+      <c r="C150" s="5" t="inlineStr">
         <is>
           <t>Heidi Bohn</t>
         </is>
       </c>
-      <c r="D150" s="4" t="inlineStr">
+      <c r="D150" s="5" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="E150" s="4" t="n">
+      <c r="E150" s="5" t="n">
         <v>164657</v>
       </c>
-      <c r="F150" s="4" t="inlineStr">
+      <c r="F150" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -9389,30 +10541,30 @@
       <c r="F159" t="inlineStr"/>
     </row>
     <row r="160">
-      <c r="A160" s="4" t="inlineStr">
+      <c r="A160" s="5" t="inlineStr">
         <is>
           <t>Korean Community Development Services Center</t>
         </is>
       </c>
-      <c r="B160" s="4" t="inlineStr">
+      <c r="B160" s="5" t="inlineStr">
         <is>
           <t>232303766</t>
         </is>
       </c>
-      <c r="C160" s="4" t="inlineStr">
+      <c r="C160" s="5" t="inlineStr">
         <is>
           <t>Don Yu</t>
         </is>
       </c>
-      <c r="D160" s="4" t="inlineStr">
+      <c r="D160" s="5" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="E160" s="4" t="n">
+      <c r="E160" s="5" t="n">
         <v>35385</v>
       </c>
-      <c r="F160" s="4" t="inlineStr">
+      <c r="F160" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -9601,30 +10753,30 @@
       <c r="F167" t="inlineStr"/>
     </row>
     <row r="168">
-      <c r="A168" s="4" t="inlineStr">
+      <c r="A168" s="5" t="inlineStr">
         <is>
           <t>Lancaster Avenue 21st Century Business Association CDC (LA21)</t>
         </is>
       </c>
-      <c r="B168" s="4" t="inlineStr">
+      <c r="B168" s="5" t="inlineStr">
         <is>
           <t>900502551</t>
         </is>
       </c>
-      <c r="C168" s="4" t="inlineStr">
+      <c r="C168" s="5" t="inlineStr">
         <is>
           <t>Kwaku Boateng</t>
         </is>
       </c>
-      <c r="D168" s="4" t="inlineStr">
+      <c r="D168" s="5" t="inlineStr">
         <is>
           <t>Exec. Director</t>
         </is>
       </c>
-      <c r="E168" s="4" t="n">
+      <c r="E168" s="5" t="n">
         <v>173500</v>
       </c>
-      <c r="F168" s="4" t="inlineStr">
+      <c r="F168" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -9865,30 +11017,30 @@
       <c r="F177" t="inlineStr"/>
     </row>
     <row r="178">
-      <c r="A178" s="4" t="inlineStr">
+      <c r="A178" s="5" t="inlineStr">
         <is>
           <t>Lower North Philadelphia CDC</t>
         </is>
       </c>
-      <c r="B178" s="4" t="inlineStr">
+      <c r="B178" s="5" t="inlineStr">
         <is>
           <t>823231994</t>
         </is>
       </c>
-      <c r="C178" s="4" t="inlineStr">
+      <c r="C178" s="5" t="inlineStr">
         <is>
           <t>Darnetta Arce</t>
         </is>
       </c>
-      <c r="D178" s="4" t="inlineStr">
+      <c r="D178" s="5" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="E178" s="4" t="n">
+      <c r="E178" s="5" t="n">
         <v>75000</v>
       </c>
-      <c r="F178" s="4" t="inlineStr">
+      <c r="F178" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -10311,30 +11463,30 @@
       <c r="F194" t="inlineStr"/>
     </row>
     <row r="195">
-      <c r="A195" s="4" t="inlineStr">
+      <c r="A195" s="5" t="inlineStr">
         <is>
           <t>Mt. Airy CDC</t>
         </is>
       </c>
-      <c r="B195" s="4" t="inlineStr">
+      <c r="B195" s="5" t="inlineStr">
         <is>
           <t>222526396</t>
         </is>
       </c>
-      <c r="C195" s="4" t="inlineStr">
+      <c r="C195" s="5" t="inlineStr">
         <is>
           <t>Philip Dawson</t>
         </is>
       </c>
-      <c r="D195" s="4" t="inlineStr">
+      <c r="D195" s="5" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="E195" s="4" t="n">
+      <c r="E195" s="5" t="n">
         <v>133900</v>
       </c>
-      <c r="F195" s="4" t="inlineStr">
+      <c r="F195" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -10575,30 +11727,30 @@
       <c r="F204" t="inlineStr"/>
     </row>
     <row r="205">
-      <c r="A205" s="4" t="inlineStr">
+      <c r="A205" s="5" t="inlineStr">
         <is>
           <t>Mt. Vernon Manor CDC</t>
         </is>
       </c>
-      <c r="B205" s="4" t="inlineStr">
+      <c r="B205" s="5" t="inlineStr">
         <is>
           <t>256084074</t>
         </is>
       </c>
-      <c r="C205" s="4" t="inlineStr">
+      <c r="C205" s="5" t="inlineStr">
         <is>
           <t>Robert Madden</t>
         </is>
       </c>
-      <c r="D205" s="4" t="inlineStr">
+      <c r="D205" s="5" t="inlineStr">
         <is>
           <t>President</t>
         </is>
       </c>
-      <c r="E205" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F205" s="4" t="inlineStr">
+      <c r="E205" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F205" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -10683,30 +11835,30 @@
       <c r="F208" t="inlineStr"/>
     </row>
     <row r="209">
-      <c r="A209" s="4" t="inlineStr">
+      <c r="A209" s="5" t="inlineStr">
         <is>
           <t>New Kensington CDC</t>
         </is>
       </c>
-      <c r="B209" s="4" t="inlineStr">
+      <c r="B209" s="5" t="inlineStr">
         <is>
           <t>222610536</t>
         </is>
       </c>
-      <c r="C209" s="4" t="inlineStr">
+      <c r="C209" s="5" t="inlineStr">
         <is>
           <t>William Mckinney</t>
         </is>
       </c>
-      <c r="D209" s="4" t="inlineStr">
+      <c r="D209" s="5" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="E209" s="4" t="n">
+      <c r="E209" s="5" t="n">
         <v>163057</v>
       </c>
-      <c r="F209" s="4" t="inlineStr">
+      <c r="F209" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -10947,30 +12099,30 @@
       <c r="F218" t="inlineStr"/>
     </row>
     <row r="219">
-      <c r="A219" s="4" t="inlineStr">
+      <c r="A219" s="5" t="inlineStr">
         <is>
           <t>Newbold CDC</t>
         </is>
       </c>
-      <c r="B219" s="4" t="inlineStr">
+      <c r="B219" s="5" t="inlineStr">
         <is>
           <t>542184458</t>
         </is>
       </c>
-      <c r="C219" s="4" t="inlineStr">
+      <c r="C219" s="5" t="inlineStr">
         <is>
           <t>Timothy Lidiak</t>
         </is>
       </c>
-      <c r="D219" s="4" t="inlineStr">
+      <c r="D219" s="5" t="inlineStr">
         <is>
           <t>President</t>
         </is>
       </c>
-      <c r="E219" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F219" s="4" t="inlineStr">
+      <c r="E219" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F219" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -11263,30 +12415,30 @@
       <c r="F230" t="inlineStr"/>
     </row>
     <row r="231">
-      <c r="A231" s="4" t="inlineStr">
+      <c r="A231" s="5" t="inlineStr">
         <is>
           <t>Nicetown CDC</t>
         </is>
       </c>
-      <c r="B231" s="4" t="inlineStr">
+      <c r="B231" s="5" t="inlineStr">
         <is>
           <t>233061705</t>
         </is>
       </c>
-      <c r="C231" s="4" t="inlineStr">
+      <c r="C231" s="5" t="inlineStr">
         <is>
           <t>Zakariyya Abdur Rahman</t>
         </is>
       </c>
-      <c r="D231" s="4" t="inlineStr">
+      <c r="D231" s="5" t="inlineStr">
         <is>
           <t>President/Ce</t>
         </is>
       </c>
-      <c r="E231" s="4" t="n">
+      <c r="E231" s="5" t="n">
         <v>183173</v>
       </c>
-      <c r="F231" s="4" t="inlineStr">
+      <c r="F231" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -11475,30 +12627,30 @@
       <c r="F238" t="inlineStr"/>
     </row>
     <row r="239">
-      <c r="A239" s="4" t="inlineStr">
+      <c r="A239" s="5" t="inlineStr">
         <is>
           <t>Old City District</t>
         </is>
       </c>
-      <c r="B239" s="4" t="inlineStr">
+      <c r="B239" s="5" t="inlineStr">
         <is>
           <t>232176305</t>
         </is>
       </c>
-      <c r="C239" s="4" t="inlineStr">
+      <c r="C239" s="5" t="inlineStr">
         <is>
           <t>Stephen Tornone</t>
         </is>
       </c>
-      <c r="D239" s="4" t="inlineStr">
+      <c r="D239" s="5" t="inlineStr">
         <is>
           <t>President</t>
         </is>
       </c>
-      <c r="E239" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F239" s="4" t="inlineStr">
+      <c r="E239" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F239" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -11583,30 +12735,30 @@
       <c r="F242" t="inlineStr"/>
     </row>
     <row r="243">
-      <c r="A243" s="4" t="inlineStr">
+      <c r="A243" s="5" t="inlineStr">
         <is>
           <t>Overbrook West Neighbors CDC</t>
         </is>
       </c>
-      <c r="B243" s="4" t="inlineStr">
+      <c r="B243" s="5" t="inlineStr">
         <is>
           <t>824449937</t>
         </is>
       </c>
-      <c r="C243" s="4" t="inlineStr">
+      <c r="C243" s="5" t="inlineStr">
         <is>
           <t>Gregory Allen</t>
         </is>
       </c>
-      <c r="D243" s="4" t="inlineStr">
+      <c r="D243" s="5" t="inlineStr">
         <is>
           <t>Founder And President</t>
         </is>
       </c>
-      <c r="E243" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F243" s="4" t="inlineStr">
+      <c r="E243" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F243" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -12003,30 +13155,30 @@
       <c r="F258" t="inlineStr"/>
     </row>
     <row r="259">
-      <c r="A259" s="4" t="inlineStr">
+      <c r="A259" s="5" t="inlineStr">
         <is>
           <t>Partnership CDC</t>
         </is>
       </c>
-      <c r="B259" s="4" t="inlineStr">
+      <c r="B259" s="5" t="inlineStr">
         <is>
           <t>232711533</t>
         </is>
       </c>
-      <c r="C259" s="4" t="inlineStr">
+      <c r="C259" s="5" t="inlineStr">
         <is>
           <t>Steven Williams</t>
         </is>
       </c>
-      <c r="D259" s="4" t="inlineStr">
+      <c r="D259" s="5" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="E259" s="4" t="n">
+      <c r="E259" s="5" t="n">
         <v>79619</v>
       </c>
-      <c r="F259" s="4" t="inlineStr">
+      <c r="F259" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -12163,30 +13315,30 @@
       <c r="F264" t="inlineStr"/>
     </row>
     <row r="265">
-      <c r="A265" s="4" t="inlineStr">
+      <c r="A265" s="5" t="inlineStr">
         <is>
           <t>Philadelphia Chinatown Development Corporation</t>
         </is>
       </c>
-      <c r="B265" s="4" t="inlineStr">
+      <c r="B265" s="5" t="inlineStr">
         <is>
           <t>237439723</t>
         </is>
       </c>
-      <c r="C265" s="4" t="inlineStr">
+      <c r="C265" s="5" t="inlineStr">
         <is>
           <t>Mr John Chin</t>
         </is>
       </c>
-      <c r="D265" s="4" t="inlineStr">
+      <c r="D265" s="5" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="E265" s="4" t="n">
+      <c r="E265" s="5" t="n">
         <v>86116</v>
       </c>
-      <c r="F265" s="4" t="inlineStr">
+      <c r="F265" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -12427,30 +13579,30 @@
       <c r="F274" t="inlineStr"/>
     </row>
     <row r="275">
-      <c r="A275" s="4" t="inlineStr">
+      <c r="A275" s="5" t="inlineStr">
         <is>
           <t>ProjectHOME</t>
         </is>
       </c>
-      <c r="B275" s="4" t="inlineStr">
+      <c r="B275" s="5" t="inlineStr">
         <is>
           <t>232555950</t>
         </is>
       </c>
-      <c r="C275" s="4" t="inlineStr">
+      <c r="C275" s="5" t="inlineStr">
         <is>
           <t>S Mary Scullion Rsm</t>
         </is>
       </c>
-      <c r="D275" s="4" t="inlineStr">
+      <c r="D275" s="5" t="inlineStr">
         <is>
           <t>President/Ed (To 07/2024)</t>
         </is>
       </c>
-      <c r="E275" s="4" t="n">
+      <c r="E275" s="5" t="n">
         <v>319389</v>
       </c>
-      <c r="F275" s="4" t="inlineStr">
+      <c r="F275" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -12691,30 +13843,30 @@
       <c r="F284" t="inlineStr"/>
     </row>
     <row r="285">
-      <c r="A285" s="4" t="inlineStr">
+      <c r="A285" s="5" t="inlineStr">
         <is>
           <t>Sister Clara Muhammad CDC</t>
         </is>
       </c>
-      <c r="B285" s="4" t="inlineStr">
+      <c r="B285" s="5" t="inlineStr">
         <is>
           <t>900405460</t>
         </is>
       </c>
-      <c r="C285" s="4" t="inlineStr">
+      <c r="C285" s="5" t="inlineStr">
         <is>
           <t>Roger Powe</t>
         </is>
       </c>
-      <c r="D285" s="4" t="inlineStr">
+      <c r="D285" s="5" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="E285" s="4" t="n">
+      <c r="E285" s="5" t="n">
         <v>8100</v>
       </c>
-      <c r="F285" s="4" t="inlineStr">
+      <c r="F285" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -12747,30 +13899,30 @@
       <c r="F286" t="inlineStr"/>
     </row>
     <row r="287">
-      <c r="A287" s="4" t="inlineStr">
+      <c r="A287" s="5" t="inlineStr">
         <is>
           <t>Smart Futures CDC</t>
         </is>
       </c>
-      <c r="B287" s="4" t="inlineStr">
+      <c r="B287" s="5" t="inlineStr">
         <is>
           <t>300263715</t>
         </is>
       </c>
-      <c r="C287" s="4" t="inlineStr">
+      <c r="C287" s="5" t="inlineStr">
         <is>
           <t>David J Mosey</t>
         </is>
       </c>
-      <c r="D287" s="4" t="inlineStr">
+      <c r="D287" s="5" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="E287" s="4" t="n">
+      <c r="E287" s="5" t="n">
         <v>224542</v>
       </c>
-      <c r="F287" s="4" t="inlineStr">
+      <c r="F287" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -13011,30 +14163,30 @@
       <c r="F296" t="inlineStr"/>
     </row>
     <row r="297">
-      <c r="A297" s="4" t="inlineStr">
+      <c r="A297" s="5" t="inlineStr">
         <is>
           <t>South Kensington Community Partners</t>
         </is>
       </c>
-      <c r="B297" s="4" t="inlineStr">
+      <c r="B297" s="5" t="inlineStr">
         <is>
           <t>222446719</t>
         </is>
       </c>
-      <c r="C297" s="4" t="inlineStr">
+      <c r="C297" s="5" t="inlineStr">
         <is>
           <t>Eileen Divringi</t>
         </is>
       </c>
-      <c r="D297" s="4" t="inlineStr">
+      <c r="D297" s="5" t="inlineStr">
         <is>
           <t>President</t>
         </is>
       </c>
-      <c r="E297" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F297" s="4" t="inlineStr">
+      <c r="E297" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F297" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -13145,30 +14297,30 @@
       <c r="F301" t="inlineStr"/>
     </row>
     <row r="302">
-      <c r="A302" s="4" t="inlineStr">
+      <c r="A302" s="5" t="inlineStr">
         <is>
           <t>Southwest CDC</t>
         </is>
       </c>
-      <c r="B302" s="4" t="inlineStr">
+      <c r="B302" s="5" t="inlineStr">
         <is>
           <t>232491247</t>
         </is>
       </c>
-      <c r="C302" s="4" t="inlineStr">
+      <c r="C302" s="5" t="inlineStr">
         <is>
           <t>Donna Henry</t>
         </is>
       </c>
-      <c r="D302" s="4" t="inlineStr">
+      <c r="D302" s="5" t="inlineStr">
         <is>
           <t>Executive Di</t>
         </is>
       </c>
-      <c r="E302" s="4" t="n">
+      <c r="E302" s="5" t="n">
         <v>96593</v>
       </c>
-      <c r="F302" s="4" t="inlineStr">
+      <c r="F302" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -13487,30 +14639,30 @@
       <c r="F314" t="inlineStr"/>
     </row>
     <row r="315">
-      <c r="A315" s="4" t="inlineStr">
+      <c r="A315" s="5" t="inlineStr">
         <is>
           <t>Tacony CDC</t>
         </is>
       </c>
-      <c r="B315" s="4" t="inlineStr">
+      <c r="B315" s="5" t="inlineStr">
         <is>
           <t>233052060</t>
         </is>
       </c>
-      <c r="C315" s="4" t="inlineStr">
+      <c r="C315" s="5" t="inlineStr">
         <is>
           <t>Georgeanne Huff Labovitz</t>
         </is>
       </c>
-      <c r="D315" s="4" t="inlineStr">
+      <c r="D315" s="5" t="inlineStr">
         <is>
           <t>President</t>
         </is>
       </c>
-      <c r="E315" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F315" s="4" t="inlineStr">
+      <c r="E315" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F315" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -13647,30 +14799,30 @@
       <c r="F320" t="inlineStr"/>
     </row>
     <row r="321">
-      <c r="A321" s="4" t="inlineStr">
+      <c r="A321" s="5" t="inlineStr">
         <is>
           <t>The Enterprise Center CDC</t>
         </is>
       </c>
-      <c r="B321" s="4" t="inlineStr">
+      <c r="B321" s="5" t="inlineStr">
         <is>
           <t>300002632</t>
         </is>
       </c>
-      <c r="C321" s="4" t="inlineStr">
+      <c r="C321" s="5" t="inlineStr">
         <is>
           <t>Della Clark</t>
         </is>
       </c>
-      <c r="D321" s="4" t="inlineStr">
+      <c r="D321" s="5" t="inlineStr">
         <is>
           <t>President</t>
         </is>
       </c>
-      <c r="E321" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F321" s="4" t="inlineStr">
+      <c r="E321" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F321" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -13859,30 +15011,30 @@
       <c r="F328" t="inlineStr"/>
     </row>
     <row r="329">
-      <c r="A329" s="4" t="inlineStr">
+      <c r="A329" s="5" t="inlineStr">
         <is>
           <t>The Maple Corporation</t>
         </is>
       </c>
-      <c r="B329" s="4" t="inlineStr">
+      <c r="B329" s="5" t="inlineStr">
         <is>
           <t>236432397</t>
         </is>
       </c>
-      <c r="C329" s="4" t="inlineStr">
+      <c r="C329" s="5" t="inlineStr">
         <is>
           <t>Jacquelyn Sims</t>
         </is>
       </c>
-      <c r="D329" s="4" t="inlineStr">
+      <c r="D329" s="5" t="inlineStr">
         <is>
           <t>President/Executive Director(sch.O)</t>
         </is>
       </c>
-      <c r="E329" s="4" t="n">
+      <c r="E329" s="5" t="n">
         <v>95007</v>
       </c>
-      <c r="F329" s="4" t="inlineStr">
+      <c r="F329" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -14149,30 +15301,30 @@
       <c r="F339" t="inlineStr"/>
     </row>
     <row r="340">
-      <c r="A340" s="4" t="inlineStr">
+      <c r="A340" s="5" t="inlineStr">
         <is>
           <t>Tioga United</t>
         </is>
       </c>
-      <c r="B340" s="4" t="inlineStr">
+      <c r="B340" s="5" t="inlineStr">
         <is>
           <t>233101958</t>
         </is>
       </c>
-      <c r="C340" s="4" t="inlineStr">
+      <c r="C340" s="5" t="inlineStr">
         <is>
           <t>David Smith</t>
         </is>
       </c>
-      <c r="D340" s="4" t="inlineStr">
+      <c r="D340" s="5" t="inlineStr">
         <is>
           <t>President</t>
         </is>
       </c>
-      <c r="E340" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F340" s="4" t="inlineStr">
+      <c r="E340" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F340" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -14257,30 +15409,30 @@
       <c r="F343" t="inlineStr"/>
     </row>
     <row r="344">
-      <c r="A344" s="4" t="inlineStr">
+      <c r="A344" s="5" t="inlineStr">
         <is>
           <t>Women's Community Revitalization Project (WCRP)</t>
         </is>
       </c>
-      <c r="B344" s="4" t="inlineStr">
+      <c r="B344" s="5" t="inlineStr">
         <is>
           <t>222840188</t>
         </is>
       </c>
-      <c r="C344" s="4" t="inlineStr">
+      <c r="C344" s="5" t="inlineStr">
         <is>
           <t>Nora Lichtash</t>
         </is>
       </c>
-      <c r="D344" s="4" t="inlineStr">
+      <c r="D344" s="5" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="E344" s="4" t="n">
+      <c r="E344" s="5" t="n">
         <v>144808</v>
       </c>
-      <c r="F344" s="4" t="inlineStr">
+      <c r="F344" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -14755,30 +15907,30 @@
       <c r="F362" t="inlineStr"/>
     </row>
     <row r="363">
-      <c r="A363" s="4" t="inlineStr">
+      <c r="A363" s="5" t="inlineStr">
         <is>
           <t>Xiente</t>
         </is>
       </c>
-      <c r="B363" s="4" t="inlineStr">
+      <c r="B363" s="5" t="inlineStr">
         <is>
           <t>239233412</t>
         </is>
       </c>
-      <c r="C363" s="4" t="inlineStr">
+      <c r="C363" s="5" t="inlineStr">
         <is>
           <t>Michelle Carrera</t>
         </is>
       </c>
-      <c r="D363" s="4" t="inlineStr">
+      <c r="D363" s="5" t="inlineStr">
         <is>
           <t>Ceo</t>
         </is>
       </c>
-      <c r="E363" s="4" t="n">
+      <c r="E363" s="5" t="n">
         <v>178453</v>
       </c>
-      <c r="F363" s="4" t="inlineStr">
+      <c r="F363" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -15019,30 +16171,30 @@
       <c r="F372" t="inlineStr"/>
     </row>
     <row r="373">
-      <c r="A373" s="4" t="inlineStr">
+      <c r="A373" s="5" t="inlineStr">
         <is>
           <t>ACHIEVEability</t>
         </is>
       </c>
-      <c r="B373" s="4" t="inlineStr">
+      <c r="B373" s="5" t="inlineStr">
         <is>
           <t>232215980</t>
         </is>
       </c>
-      <c r="C373" s="4" t="inlineStr">
+      <c r="C373" s="5" t="inlineStr">
         <is>
           <t>Jamila Harris Morrison</t>
         </is>
       </c>
-      <c r="D373" s="4" t="inlineStr">
+      <c r="D373" s="5" t="inlineStr">
         <is>
           <t>Executive Di</t>
         </is>
       </c>
-      <c r="E373" s="4" t="n">
+      <c r="E373" s="5" t="n">
         <v>176423</v>
       </c>
-      <c r="F373" s="4" t="inlineStr">
+      <c r="F373" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -15283,30 +16435,30 @@
       <c r="F382" t="inlineStr"/>
     </row>
     <row r="383">
-      <c r="A383" s="4" t="inlineStr">
+      <c r="A383" s="5" t="inlineStr">
         <is>
           <t>Fairmount CDC</t>
         </is>
       </c>
-      <c r="B383" s="4" t="inlineStr">
+      <c r="B383" s="5" t="inlineStr">
         <is>
           <t>233094818</t>
         </is>
       </c>
-      <c r="C383" s="4" t="inlineStr">
+      <c r="C383" s="5" t="inlineStr">
         <is>
           <t>Patrick Sherlock</t>
         </is>
       </c>
-      <c r="D383" s="4" t="inlineStr">
+      <c r="D383" s="5" t="inlineStr">
         <is>
           <t>Exec Directo</t>
         </is>
       </c>
-      <c r="E383" s="4" t="n">
+      <c r="E383" s="5" t="n">
         <v>74938</v>
       </c>
-      <c r="F383" s="4" t="inlineStr">
+      <c r="F383" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -15703,30 +16855,30 @@
       <c r="F398" t="inlineStr"/>
     </row>
     <row r="399">
-      <c r="A399" s="4" t="inlineStr">
+      <c r="A399" s="5" t="inlineStr">
         <is>
           <t>Francisville Neighborhood Development Corporation</t>
         </is>
       </c>
-      <c r="B399" s="4" t="inlineStr">
+      <c r="B399" s="5" t="inlineStr">
         <is>
           <t>571164331</t>
         </is>
       </c>
-      <c r="C399" s="4" t="inlineStr">
+      <c r="C399" s="5" t="inlineStr">
         <is>
           <t>Penelope Giles</t>
         </is>
       </c>
-      <c r="D399" s="4" t="inlineStr">
+      <c r="D399" s="5" t="inlineStr">
         <is>
           <t>President</t>
         </is>
       </c>
-      <c r="E399" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F399" s="4" t="inlineStr">
+      <c r="E399" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F399" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -16201,30 +17353,30 @@
       <c r="F417" t="inlineStr"/>
     </row>
     <row r="418">
-      <c r="A418" s="4" t="inlineStr">
+      <c r="A418" s="5" t="inlineStr">
         <is>
           <t>Spring Garden CDC</t>
         </is>
       </c>
-      <c r="B418" s="4" t="inlineStr">
+      <c r="B418" s="5" t="inlineStr">
         <is>
           <t>232772462</t>
         </is>
       </c>
-      <c r="C418" s="4" t="inlineStr">
+      <c r="C418" s="5" t="inlineStr">
         <is>
           <t>Patricia Freeland</t>
         </is>
       </c>
-      <c r="D418" s="4" t="inlineStr">
+      <c r="D418" s="5" t="inlineStr">
         <is>
           <t>President/Board Member</t>
         </is>
       </c>
-      <c r="E418" s="4" t="n">
+      <c r="E418" s="5" t="n">
         <v>18750</v>
       </c>
-      <c r="F418" s="4" t="inlineStr">
+      <c r="F418" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -16309,30 +17461,30 @@
       <c r="F421" t="inlineStr"/>
     </row>
     <row r="422">
-      <c r="A422" s="4" t="inlineStr">
+      <c r="A422" s="5" t="inlineStr">
         <is>
           <t>Allegheny West Foundation</t>
         </is>
       </c>
-      <c r="B422" s="4" t="inlineStr">
+      <c r="B422" s="5" t="inlineStr">
         <is>
           <t>231924667</t>
         </is>
       </c>
-      <c r="C422" s="4" t="inlineStr">
+      <c r="C422" s="5" t="inlineStr">
         <is>
           <t>Ronald Hinton</t>
         </is>
       </c>
-      <c r="D422" s="4" t="inlineStr">
+      <c r="D422" s="5" t="inlineStr">
         <is>
           <t>President/Exec Dir</t>
         </is>
       </c>
-      <c r="E422" s="4" t="n">
+      <c r="E422" s="5" t="n">
         <v>124604</v>
       </c>
-      <c r="F422" s="4" t="inlineStr">
+      <c r="F422" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -16573,30 +17725,30 @@
       <c r="F431" t="inlineStr"/>
     </row>
     <row r="432">
-      <c r="A432" s="4" t="inlineStr">
+      <c r="A432" s="5" t="inlineStr">
         <is>
           <t>Village of Arts and Humanities</t>
         </is>
       </c>
-      <c r="B432" s="4" t="inlineStr">
+      <c r="B432" s="5" t="inlineStr">
         <is>
           <t>223045318</t>
         </is>
       </c>
-      <c r="C432" s="4" t="inlineStr">
+      <c r="C432" s="5" t="inlineStr">
         <is>
           <t>Ineda Elmore Stratton</t>
         </is>
       </c>
-      <c r="D432" s="4" t="inlineStr">
+      <c r="D432" s="5" t="inlineStr">
         <is>
           <t>Executive Director Thru 7/11/24</t>
         </is>
       </c>
-      <c r="E432" s="4" t="n">
+      <c r="E432" s="5" t="n">
         <v>119539</v>
       </c>
-      <c r="F432" s="4" t="inlineStr">
+      <c r="F432" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -16811,30 +17963,30 @@
       <c r="F440" t="inlineStr"/>
     </row>
     <row r="441">
-      <c r="A441" s="4" t="inlineStr">
+      <c r="A441" s="5" t="inlineStr">
         <is>
           <t>Faith CDC</t>
         </is>
       </c>
-      <c r="B441" s="4" t="inlineStr">
+      <c r="B441" s="5" t="inlineStr">
         <is>
           <t>43673651</t>
         </is>
       </c>
-      <c r="C441" s="4" t="inlineStr">
+      <c r="C441" s="5" t="inlineStr">
         <is>
           <t>Mehboob Khan</t>
         </is>
       </c>
-      <c r="D441" s="4" t="inlineStr">
+      <c r="D441" s="5" t="inlineStr">
         <is>
           <t>President</t>
         </is>
       </c>
-      <c r="E441" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F441" s="4" t="inlineStr">
+      <c r="E441" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F441" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -17127,60 +18279,60 @@
       <c r="F452" t="inlineStr"/>
     </row>
     <row r="453">
-      <c r="A453" s="4" t="inlineStr">
+      <c r="A453" s="5" t="inlineStr">
         <is>
           <t>Mt. Airy Village Development Corporation</t>
         </is>
       </c>
-      <c r="B453" s="4" t="inlineStr">
+      <c r="B453" s="5" t="inlineStr">
         <is>
           <t>260898815</t>
         </is>
       </c>
-      <c r="C453" s="4" t="inlineStr">
+      <c r="C453" s="5" t="inlineStr">
         <is>
           <t>Isaac Ewell</t>
         </is>
       </c>
-      <c r="D453" s="4" t="inlineStr">
+      <c r="D453" s="5" t="inlineStr">
         <is>
           <t>Chair/President</t>
         </is>
       </c>
-      <c r="E453" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F453" s="4" t="inlineStr">
+      <c r="E453" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F453" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
     <row r="454">
-      <c r="A454" s="4" t="inlineStr">
+      <c r="A454" s="5" t="inlineStr">
         <is>
           <t>West Oak Lane CDC</t>
         </is>
       </c>
-      <c r="B454" s="4" t="inlineStr">
+      <c r="B454" s="5" t="inlineStr">
         <is>
           <t>232142704</t>
         </is>
       </c>
-      <c r="C454" s="4" t="inlineStr">
+      <c r="C454" s="5" t="inlineStr">
         <is>
           <t>Donald T Stafford</t>
         </is>
       </c>
-      <c r="D454" s="4" t="inlineStr">
+      <c r="D454" s="5" t="inlineStr">
         <is>
           <t>Director</t>
         </is>
       </c>
-      <c r="E454" s="4" t="n">
+      <c r="E454" s="5" t="n">
         <v>46501</v>
       </c>
-      <c r="F454" s="4" t="inlineStr">
+      <c r="F454" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -17265,30 +18417,30 @@
       <c r="F457" t="inlineStr"/>
     </row>
     <row r="458">
-      <c r="A458" s="4" t="inlineStr">
+      <c r="A458" s="5" t="inlineStr">
         <is>
           <t>Roxborough Development Corporation</t>
         </is>
       </c>
-      <c r="B458" s="4" t="inlineStr">
+      <c r="B458" s="5" t="inlineStr">
         <is>
           <t>232705347</t>
         </is>
       </c>
-      <c r="C458" s="4" t="inlineStr">
+      <c r="C458" s="5" t="inlineStr">
         <is>
           <t>Jax Cusack</t>
         </is>
       </c>
-      <c r="D458" s="4" t="inlineStr">
+      <c r="D458" s="5" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="E458" s="4" t="n">
+      <c r="E458" s="5" t="n">
         <v>92900</v>
       </c>
-      <c r="F458" s="4" t="inlineStr">
+      <c r="F458" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -17581,30 +18733,30 @@
       <c r="F469" t="inlineStr"/>
     </row>
     <row r="470">
-      <c r="A470" s="4" t="inlineStr">
+      <c r="A470" s="5" t="inlineStr">
         <is>
           <t>Yorktown CDC</t>
         </is>
       </c>
-      <c r="B470" s="4" t="inlineStr">
+      <c r="B470" s="5" t="inlineStr">
         <is>
           <t>232642355</t>
         </is>
       </c>
-      <c r="C470" s="4" t="inlineStr">
+      <c r="C470" s="5" t="inlineStr">
         <is>
           <t>Renee V Drayton</t>
         </is>
       </c>
-      <c r="D470" s="4" t="inlineStr">
+      <c r="D470" s="5" t="inlineStr">
         <is>
           <t>President</t>
         </is>
       </c>
-      <c r="E470" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F470" s="4" t="inlineStr">
+      <c r="E470" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F470" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -17793,30 +18945,30 @@
       <c r="F477" t="inlineStr"/>
     </row>
     <row r="478">
-      <c r="A478" s="4" t="inlineStr">
+      <c r="A478" s="5" t="inlineStr">
         <is>
           <t>Tenth Memorial Non-Profit Development Corporation</t>
         </is>
       </c>
-      <c r="B478" s="4" t="inlineStr">
+      <c r="B478" s="5" t="inlineStr">
         <is>
           <t>222538855</t>
         </is>
       </c>
-      <c r="C478" s="4" t="inlineStr">
+      <c r="C478" s="5" t="inlineStr">
         <is>
           <t>Rev William B Moore</t>
         </is>
       </c>
-      <c r="D478" s="4" t="inlineStr">
+      <c r="D478" s="5" t="inlineStr">
         <is>
           <t>President</t>
         </is>
       </c>
-      <c r="E478" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F478" s="4" t="inlineStr">
+      <c r="E478" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F478" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -17979,30 +19131,30 @@
       <c r="F484" t="inlineStr"/>
     </row>
     <row r="485">
-      <c r="A485" s="4" t="inlineStr">
+      <c r="A485" s="5" t="inlineStr">
         <is>
           <t>Olde Kensington Redevelopment Corporation</t>
         </is>
       </c>
-      <c r="B485" s="4" t="inlineStr">
+      <c r="B485" s="5" t="inlineStr">
         <is>
           <t>834158522</t>
         </is>
       </c>
-      <c r="C485" s="4" t="inlineStr">
+      <c r="C485" s="5" t="inlineStr">
         <is>
           <t>John Williams</t>
         </is>
       </c>
-      <c r="D485" s="4" t="inlineStr">
+      <c r="D485" s="5" t="inlineStr">
         <is>
           <t>President</t>
         </is>
       </c>
-      <c r="E485" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F485" s="4" t="inlineStr">
+      <c r="E485" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F485" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -18035,30 +19187,30 @@
       <c r="F486" t="inlineStr"/>
     </row>
     <row r="487">
-      <c r="A487" s="4" t="inlineStr">
+      <c r="A487" s="5" t="inlineStr">
         <is>
           <t>Kensington Area Revitalization Project</t>
         </is>
       </c>
-      <c r="B487" s="4" t="inlineStr">
+      <c r="B487" s="5" t="inlineStr">
         <is>
           <t>844037072</t>
         </is>
       </c>
-      <c r="C487" s="4" t="inlineStr">
+      <c r="C487" s="5" t="inlineStr">
         <is>
           <t>Marc D Collazzo</t>
         </is>
       </c>
-      <c r="D487" s="4" t="inlineStr">
+      <c r="D487" s="5" t="inlineStr">
         <is>
           <t>Executive Director</t>
         </is>
       </c>
-      <c r="E487" s="4" t="n">
+      <c r="E487" s="5" t="n">
         <v>150719</v>
       </c>
-      <c r="F487" s="4" t="inlineStr">
+      <c r="F487" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -18303,7 +19455,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -37470,7 +38622,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -41528,7 +42680,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -57494,7 +58646,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -69287,7 +70439,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -70566,7 +71718,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -70579,7 +71731,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Corridor — Philadelphia CDC dataset</t>
         </is>

</xml_diff>

<commit_message>
fix(web): remove personal name from public-facing site and spreadsheet
Renamed the "Ben roster" source label to "Research roster" (data/
cdc_roster.csv, output/roster.csv, both flow into dataset.json and the
xlsx), which also matters because org.source renders directly in the
site's "Source note (<source>)" callout on org detail pages. Removed
the same name from the About page, the Map page's footnote, the xlsx
About sheet's sourcing writeup, the ED Timeline sheet's note row, and
one org's research note that mentioned it directly.
</commit_message>
<xml_diff>
--- a/output/corridor_dataset.xlsx
+++ b/output/corridor_dataset.xlsx
@@ -717,7 +717,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -993,7 +993,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1488,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>Per Ben's research, this org's activity continued as Park to Broad Arts &amp; Business District (already tracked separately on this roster).</t>
+          <t>Per project research, this org's activity continued as Park to Broad Arts &amp; Business District (already tracked separately on this roster).</t>
         </is>
       </c>
     </row>
@@ -1740,7 +1740,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -1943,7 +1943,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -2038,7 +2038,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -2058,7 +2058,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -2098,7 +2098,7 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -2147,7 +2147,7 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -2252,7 +2252,7 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -2357,7 +2357,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -2534,7 +2534,7 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -2658,7 +2658,7 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -2819,7 +2819,7 @@
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -2925,7 +2925,7 @@
       <c r="N58" s="3" t="inlineStr"/>
       <c r="R58" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -3036,7 +3036,7 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -3167,7 +3167,7 @@
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -3248,7 +3248,7 @@
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -3367,7 +3367,7 @@
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -3431,7 +3431,7 @@
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -3482,7 +3482,7 @@
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -3503,7 +3503,7 @@
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -3579,7 +3579,7 @@
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -3635,7 +3635,7 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -3731,7 +3731,7 @@
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -3795,7 +3795,7 @@
       </c>
       <c r="R79" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -3840,7 +3840,7 @@
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -3899,7 +3899,7 @@
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -4011,7 +4011,7 @@
       </c>
       <c r="R85" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -4072,7 +4072,7 @@
       </c>
       <c r="R86" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -4309,7 +4309,7 @@
       </c>
       <c r="R91" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -4404,7 +4404,7 @@
       </c>
       <c r="R93" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -4449,7 +4449,7 @@
       </c>
       <c r="R94" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -4514,7 +4514,7 @@
       </c>
       <c r="R95" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -4558,7 +4558,7 @@
       </c>
       <c r="R96" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
       <c r="S96" t="inlineStr">
@@ -4804,7 +4804,7 @@
       </c>
       <c r="R101" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -4889,7 +4889,7 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>Ben roster</t>
+          <t>Research roster</t>
         </is>
       </c>
     </row>
@@ -12322,7 +12322,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NOTE: sample of 20 organizations drawn at random from the full roster (data/ed_timeline_sample.txt). Years come primarily from Ben's own research; where that data stops before the present and the automated pipeline found a different named current executive, that name is added with its start year marked unconfirmed. A blank cell means the organization existed but no leader is confirmed for that year, not that the seat was vacant.</t>
+          <t>NOTE: sample of 20 organizations drawn at random from the full roster (data/ed_timeline_sample.txt). Years come primarily from direct research; where that data stops before the present and the automated pipeline found a different named current executive, that name is added with its start year marked unconfirmed. A blank cell means the organization existed but no leader is confirmed for that year, not that the seat was vacant.</t>
         </is>
       </c>
     </row>
@@ -81828,7 +81828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A60"/>
+  <dimension ref="A1:A61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="92" customWidth="1" min="1" max="1"/>
@@ -81901,336 +81901,343 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  organizations, founding to present, in the format of Ben's BID Exec Director Timelines.</t>
+          <t xml:space="preserve">  organizations, founding to present, in the format of a BID executive-director timeline</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Leadership: the full current officer and board roster per organization, from IRS Form 990 Part VII.</t>
+          <t xml:space="preserve">  reference used for this project.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Titles carrying a '(To MM/YYYY)' note mark an officer who was on the way out — a recorded transition.</t>
+          <t>Leadership: the full current officer and board roster per organization, from IRS Form 990 Part VII.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Financial History: revenue, expenses, assets, staff, and officer pay per organization-year.</t>
+          <t xml:space="preserve">  Titles carrying a '(To MM/YYYY)' note mark an officer who was on the way out — a recorded transition.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Tax Credit: participation in the City of Philadelphia CDC Tax Credit program by report year,</t>
+          <t>Financial History: revenue, expenses, assets, staff, and officer pay per organization-year.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  with the year each organization entered and its annual contribution. Source PDFs: phila.gov.</t>
+          <t>Tax Credit: participation in the City of Philadelphia CDC Tax Credit program by report year,</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>990 PDFs: a direct link to every Form 990 document on file, by organization and year.</t>
+          <t xml:space="preserve">  with the year each organization entered and its annual contribution. Source PDFs: phila.gov.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>News &amp; Sources: recent articles per organization, including a dedicated Philadelphia Inquirer</t>
+          <t>990 PDFs: a direct link to every Form 990 document on file, by organization and year.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  search alongside general Google News coverage and leadership-change coverage.</t>
+          <t>News &amp; Sources: recent articles per organization, including a dedicated Philadelphia Inquirer</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t xml:space="preserve">  search alongside general Google News coverage and leadership-change coverage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>Signals: organizations ranked by how much their record suggests leadership instability.</t>
         </is>
       </c>
     </row>
-    <row r="21"/>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>WHERE EVERY PIECE OF DATA CAME FROM</t>
-        </is>
-      </c>
-    </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>The roster itself: three separate rounds, each tagged in the Roster sheet's 'Roster source' column.</t>
+          <t>WHERE EVERY PIECE OF DATA CAME FROM</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - 'Ben roster' (70 orgs): Ben's original hand-compiled list, plus his own follow-up research —</t>
+          <t>The roster itself: three separate rounds, each tagged in the Roster sheet's 'Roster source' column.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">    years active, full historical leadership with tenure ranges, mission statements, addresses,</t>
+          <t xml:space="preserve">  - 'Research roster' (70 orgs): the project's original hand-compiled list, plus follow-up</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    and notes — folded into this roster's Notes/Address columns and into the Leadership and</t>
+          <t xml:space="preserve">    research — years active, full historical leadership with tenure ranges, mission statements,</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ED Timeline sheets.</t>
+          <t xml:space="preserve">    addresses, and notes — folded into this roster's Notes/Address columns and into the</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - 'City CDC program' (9 orgs): the City of Philadelphia's own list of CDC Tax Credit program</t>
+          <t xml:space="preserve">    Leadership and ED Timeline sheets.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">    participants (phila.gov).</t>
+          <t xml:space="preserve">  - 'City CDC program' (9 orgs): the City of Philadelphia's own list of CDC Tax Credit program</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - 'Temple archives' (29 orgs): read directly from 13 PDF finding aids Ben obtained from Temple</t>
+          <t xml:space="preserve">    participants (phila.gov).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">    University's Special Collections Research Center (library.temple.edu/scrc) — the Philadelphia</t>
+          <t xml:space="preserve">  - 'Temple archives' (29 orgs): read directly from 13 PDF finding aids from Temple University's</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Association of Community Development Corporations' own member records (SCRC 241), plus</t>
+          <t xml:space="preserve">    Special Collections Research Center (library.temple.edu/scrc) — the Philadelphia Association</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">    standalone collections for Germantown Settlement, Weccacoe Development Association, Olde</t>
+          <t xml:space="preserve">    of Community Development Corporations' own member records (SCRC 241), plus standalone</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Kensington Redevelopment Corporation/Senior Housing Associates, West Philadelphia Corporation,</t>
+          <t xml:space="preserve">    collections for Germantown Settlement, Weccacoe Development Association, Olde Kensington</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    Kensington Action Now, and the Regional Council of Neighborhood Organizations.</t>
+          <t xml:space="preserve">    Redevelopment Corporation/Senior Housing Associates, West Philadelphia Corporation, Kensington</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - 'PACDC member list' (1 org) and 'Regional Foundation partners page' (1 org): cross-referenced</t>
+          <t xml:space="preserve">    Action Now, and the Regional Council of Neighborhood Organizations.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">    PACDC's own FY25 Annual Report (pacdc.org) and the Regional Foundation's partners page</t>
+          <t xml:space="preserve">  - 'PACDC member list' (1 org) and 'Regional Foundation partners page' (1 org): cross-referenced</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    (regionalfoundation.org) against the existing roster to find CDCs not yet tracked.</t>
+          <t xml:space="preserve">    PACDC's own FY25 Annual Report (pacdc.org) and the Regional Foundation's partners page</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Two more ('Ben roster'): Urban Resources Development Corporation and Eastwick United CDC,</t>
+          <t xml:space="preserve">    (regionalfoundation.org) against the existing roster to find CDCs not yet tracked.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">    surfaced from Ben's own research CSV and independently verified before adding.</t>
+          <t xml:space="preserve">  - Two more ('Research roster'): Urban Resources Development Corporation and Eastwick United CDC,</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Checked but yielded no new organizations: shelterforce.org (national context, no Philadelphia-</t>
+          <t xml:space="preserve">    surfaced from further research and independently verified before adding.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">    specific CDC names).</t>
+          <t xml:space="preserve">  - Checked but yielded no new organizations: shelterforce.org (national context, no Philadelphia-</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Financials, EIN matching, current officers, and Form 990 links: the ProPublica Nonprofit Explorer</t>
+          <t xml:space="preserve">    specific CDC names).</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">  API (projects.propublica.org/nonprofits), matched to each roster name by fuzzy string match,</t>
+          <t>Financials, EIN matching, current officers, and Form 990 links: the ProPublica Nonprofit Explorer</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">  scored and flagged by confidence rather than guessed. Historical (year-by-year) director names</t>
+          <t xml:space="preserve">  API (projects.propublica.org/nonprofits), matched to each roster name by fuzzy string match,</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">  are NOT available this way — see the limitation note below.</t>
+          <t xml:space="preserve">  scored and flagged by confidence rather than guessed. Historical (year-by-year) director names</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>News coverage: Google News search per organization, plus a Philadelphia-Inquirer-specific</t>
+          <t xml:space="preserve">  are NOT available this way — see the limitation note below.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">  site-scoped search so real Inquirer coverage isn't crowded out by more numerous generic sources.</t>
+          <t>News coverage: Google News search per organization, plus a Philadelphia-Inquirer-specific</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Tax-credit participation: the City of Philadelphia's own annual CDC Tax Credit program reports</t>
+          <t xml:space="preserve">  site-scoped search so real Inquirer coverage isn't crowded out by more numerous generic sources.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>Tax-credit participation: the City of Philadelphia's own annual CDC Tax Credit program reports</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t xml:space="preserve">  (phila.gov), parsed from the source PDFs (2015, 2019, 2020 and other available years).</t>
         </is>
       </c>
     </row>
-    <row r="51"/>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>THE HONEST LIMITATION</t>
-        </is>
-      </c>
-    </row>
+    <row r="52"/>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Executive directors and boards from ProPublica are current as of each organization's latest Form</t>
+          <t>THE HONEST LIMITATION</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">  990, not a full year-by-year history — as of 2026 there is no free, lightweight way to pull</t>
+          <t>Executive directors and boards from ProPublica are current as of each organization's latest Form</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">  historical Form 990 Part VII names at scale (the AWS 990 mirror was retired, the IRS per-file</t>
+          <t xml:space="preserve">  990, not a full year-by-year history — as of 2026 there is no free, lightweight way to pull</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">  XML URLs 404, and ProPublica blocks scripted PDF downloads). Where a fuller history exists, it's</t>
+          <t xml:space="preserve">  historical Form 990 Part VII names at scale (the AWS 990 mirror was retired, the IRS per-file</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">  because Ben's own research found it by hand — that's what powers the Leadership tenure ranges</t>
+          <t xml:space="preserve">  XML URLs 404, and ProPublica blocks scripted PDF downloads). Where a fuller history exists, it's</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">  in the Roster notes and the ED Timeline sheet, not an automated source. The pay-shift years flag</t>
+          <t xml:space="preserve">  because direct research found it by hand — that's what powers the Leadership tenure ranges</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">  when a change most likely happened from officer-compensation swings; the news links are where</t>
+          <t xml:space="preserve">  in the Roster notes and the ED Timeline sheet, not an automated source. The pay-shift years flag</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  when a change most likely happened from officer-compensation swings; the news links are where</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
         <is>
           <t xml:space="preserve">  the actual named change is reported.</t>
         </is>

</xml_diff>